<commit_message>
Example file: rows the system codes the way a customer writes them
The old primer.xlsx had made-up rows with too few characteristics: one of 8 went to auto
(paper at 32 %), the first thing a visitor sees after «Взять пример». The new one is made by
scripts/make_primer.py from rows of the organizers' files and the real food specification,
in the template's columns: 11 rows, 11/11 exact codes, 10 in auto, all right, in two live
runs. The kefir stays for review on purpose (two codes of one name), the security service
shows that services are coded too. Its reference is dataset/primer/primer_reference.jsonl.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/primer.xlsx
+++ b/frontend/public/primer.xlsx
@@ -420,14 +420,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -463,21 +463,21 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Бумага для офисной техники А4</t>
+          <t>Ноутбук</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Плотность 80 г/м2, 500 листов в пачке, белизна не менее 146 %</t>
+          <t>Диагональ экрана: не менее 15.6 дюйма; оперативная память 16 ГБ; тип накопителя SSD; разрешение экрана Full HD; количество ядер процессора 4</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>пачка</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -486,12 +486,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Мыло туалетное твердое</t>
+          <t>Мышь компьютерная</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Масса 100 г, без отдушки</t>
+          <t>Тип подключения: беспроводной; интерфейс USB; питание от аккумулятора; мультифункциональные клавиши: да</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -500,7 +500,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -509,21 +509,21 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Перчатки смотровые нитриловые неопудренные</t>
+          <t>Клавиатура</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Размер M, нестерильные</t>
+          <t>Тип подключения: проводная; полноразмерная; интерфейс USB; длина кабеля 1,6 м</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>пара</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>200</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -532,12 +532,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Шприц инъекционный трехкомпонентный</t>
+          <t>Тетрадь ученическая школьная</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Объем 5 мл, с иглой</t>
+          <t>Линовка: линейка; 12 листов</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="6">
@@ -555,21 +555,21 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Кефир</t>
+          <t>Папка картонная</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Массовая доля жира 2,5 %, упаковка 1 л</t>
+          <t>Формат А3; папка-обложка без скоросшивателя</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>л</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
@@ -578,21 +578,21 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Ноутбук</t>
+          <t>Полотенце бумажное</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Диагональ экрана 15.6 дюйм, оперативная память 16 ГБ, SSD 512 ГБ</t>
+          <t>Форма выпуска: лист; 50 листов в упаковке</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>упак</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>2</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8">
@@ -601,12 +601,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Картридж для лазерного принтера</t>
+          <t>Лампа светодиодная</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Черный, ресурс не менее 1600 страниц</t>
+          <t>Двухцокольная; мощность 10 Вт; цоколь G23; цветовая температура 2700 К</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9">
@@ -624,12 +624,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Стол письменный</t>
+          <t>Телевизор</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Длина 1200 мм, ширина 600 мм, ЛДСП</t>
+          <t>Тип экрана QLED; разрешение 8K UHD; диагональ 40 дюймов; Smart TV: да; 3D-экран: да</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -638,7 +638,76 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Масло сливочное</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Сладко-сливочное, Крестьянское, высший сорт, несоленое</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>кг</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Кефир</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Тип молочного сырья: нормализованное молоко; 2,5 процента</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>л</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Услуги частной охраны (выставление поста охраны)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Охрана имущества и обеспечение пропускного режима на объектах с требованиями к антитеррористической защищенности</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>усл. ед</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>